<commit_message>
Add locations template, RTL support, and location auto-block
Migrates the business overview, help-and-support, and locations pages
(plus their Arabic ar-ae versions) into AEM.

- New locations template: hero-text (text-only page intro) + cards-location
  (branch/partner list) + reused cards-support + app-promo.
- cards-location auto-block in scripts.js groups the location finder's loose
  paragraphs into cards (name/address/phone), handling English "More" and
  Arabic "أكثر" boundaries; skips the non-migratable Google Map.
- taqa-cleanup transformer strips the Google Maps widget so its chrome
  doesn't leak into imported content.
- RTL: scripts.js sets dir=rtl/lang=ar for /ar-ae/ paths; global + header
  RTL CSS mirrors the layout for Arabic pages.
- business/overview reuses the residential (spotlight/USP/news) template.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-help-and-support.report.xlsx
+++ b/tools/importer/reports/import-help-and-support.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="103">
   <si>
     <t>_reportFile</t>
   </si>
@@ -109,25 +109,205 @@
     <t>https://www.nileair.com/travelling-pets</t>
   </si>
   <si>
+    <t>addc/en-us/business/overview.report.json</t>
+  </si>
+  <si>
+    <t>["hero-residential","cards-usp-overlay","cards-usp-overlay","cards-news"]</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/overview</t>
+  </si>
+  <si>
+    <t>residential</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:29:01.841Z</t>
+  </si>
+  <si>
+    <t>TAQA Distribution</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/overview</t>
+  </si>
+  <si>
+    <t>addc/en-us/residential/overview.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/residential/overview</t>
+  </si>
+  <si>
+    <t>2026-09-17T06:08:10.043Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/residential/overview</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/account-management-and-bills.report.json</t>
+  </si>
+  <si>
+    <t>["hero-support","cards-quicklink","accordion-faq","carousel-tips","carousel-tips","cards-support"]</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/account-management-and-bills</t>
+  </si>
+  <si>
+    <t>help-and-support</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:51:35.765Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/account-management-and-bills</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/connection-of-water-services.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/connection-of-water-services</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:51:51.851Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/connection-of-water-services</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/customer-care.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/customer-care</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:51:42.220Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/customer-care</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/extension-and-connection-of-electricity-services.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/extension-and-connection-of-electricity-services</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:51:22.714Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/extension-and-connection-of-electricity-services</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/transfer-and-removal-of-electricity-services.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/transfer-and-removal-of-electricity-services</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:51:28.420Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/transfer-and-removal-of-electricity-services</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/account-management-and-bills.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/account-management-and-bills</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:27:16.806Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/help-and-support/account-management-and-bills</t>
+  </si>
+  <si>
     <t>addc/en-us/business/help-and-support/certificates.report.json</t>
   </si>
   <si>
-    <t>["hero-support","cards-quicklink","accordion-faq","carousel-tips","carousel-tips","cards-support"]</t>
-  </si>
-  <si>
     <t>addc/en-us/business/help-and-support/certificates</t>
   </si>
   <si>
-    <t>help-and-support</t>
-  </si>
-  <si>
     <t>2026-09-16T08:55:32.399Z</t>
   </si>
   <si>
-    <t>TAQA Distribution</t>
-  </si>
-  <si>
     <t>https://taqadistribution.com/addc/en-us/business/help-and-support/certificates</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/connection-of-water-services.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/connection-of-water-services</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:27:35.020Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/help-and-support/connection-of-water-services</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/customer-care.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/customer-care</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:27:25.397Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/help-and-support/customer-care</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/extension-and-connection-of-electricity-services.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/extension-and-connection-of-electricity-services</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:26:59.985Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/help-and-support/extension-and-connection-of-electricity-services</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/transfer-and-removal-of-electricity-services.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/help-and-support/transfer-and-removal-of-electricity-services</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:27:08.178Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/help-and-support/transfer-and-removal-of-electricity-services</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/locations/branches.report.json</t>
+  </si>
+  <si>
+    <t>["hero-text","cards-support"]</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/locations/branches</t>
+  </si>
+  <si>
+    <t>locations</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:47:20.889Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/locations/branches</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/locations/partners.report.json</t>
+  </si>
+  <si>
+    <t>addc/en-us/business/locations/partners</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:47:29.304Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/business/locations/partners</t>
   </si>
   <si>
     <t>addc/en-us/residential/help-and-support/transfer-and-removal-of-electricity-services.report.json</t>
@@ -528,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -720,6 +900,370 @@
         <v>42</v>
       </c>
     </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>37</v>
+      </c>
+      <c r="H10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G12" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" t="s">
+        <v>37</v>
+      </c>
+      <c r="H15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" t="s">
+        <v>83</v>
+      </c>
+      <c r="G17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" t="s">
+        <v>87</v>
+      </c>
+      <c r="G18" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19" t="s">
+        <v>37</v>
+      </c>
+      <c r="H19" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" t="s">
+        <v>97</v>
+      </c>
+      <c r="G20" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" t="s">
+        <v>101</v>
+      </c>
+      <c r="G21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H21" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix nav mega-menu leaf links not navigating on left-click
The nav-section click handler called preventDefault() for any click inside
a section that has a submenu whenever the section had no top-level <a>
trigger. Menu-only triggers like 'Help & Support' are delivered by DA as a
<p> (not a link), so every click in that section — including real leaf
links in the dropdown — was blocked; left-click did nothing while
'open in new tab' (which bypasses JS) still worked.

Only treat a click as a menu toggle when it lands on the section's trigger
element itself (top <a>/<p>/.nav-drop-toggle). Clicks on links deeper in
the submenu now navigate normally. Verified: leaf links navigate on
left-click and the trigger still toggles the mega-menu.

Also includes the rebuilt help-and-support import bundle (current
transformer) from the Arabic certificates migration.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-help-and-support.report.xlsx
+++ b/tools/importer/reports/import-help-and-support.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="119">
   <si>
     <t>_reportFile</t>
   </si>
@@ -109,22 +109,34 @@
     <t>https://www.nileair.com/travelling-pets</t>
   </si>
   <si>
+    <t>addc/ar-ae/business/overview.report.json</t>
+  </si>
+  <si>
+    <t>["hero-residential","cards-usp-overlay","cards-usp-overlay","cards-news"]</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/overview</t>
+  </si>
+  <si>
+    <t>residential</t>
+  </si>
+  <si>
+    <t>2026-09-22T10:29:45.192Z</t>
+  </si>
+  <si>
+    <t>TAQA Distribution</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/overview</t>
+  </si>
+  <si>
     <t>addc/en-us/business/overview.report.json</t>
   </si>
   <si>
-    <t>["hero-residential","cards-usp-overlay","cards-usp-overlay","cards-news"]</t>
-  </si>
-  <si>
     <t>addc/en-us/business/overview</t>
   </si>
   <si>
-    <t>residential</t>
-  </si>
-  <si>
-    <t>2026-09-22T06:29:01.841Z</t>
-  </si>
-  <si>
-    <t>TAQA Distribution</t>
+    <t>2026-09-22T10:29:29.986Z</t>
   </si>
   <si>
     <t>https://taqadistribution.com/addc/en-us/business/overview</t>
@@ -136,7 +148,7 @@
     <t>addc/en-us/residential/overview</t>
   </si>
   <si>
-    <t>2026-09-17T06:08:10.043Z</t>
+    <t>2026-09-22T10:29:38.734Z</t>
   </si>
   <si>
     <t>https://taqadistribution.com/addc/en-us/residential/overview</t>
@@ -160,6 +172,18 @@
     <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/account-management-and-bills</t>
   </si>
   <si>
+    <t>addc/ar-ae/business/help-and-support/certificates.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/help-and-support/certificates</t>
+  </si>
+  <si>
+    <t>2026-09-22T11:35:27.674Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/certificates</t>
+  </si>
+  <si>
     <t>addc/ar-ae/business/help-and-support/connection-of-water-services.report.json</t>
   </si>
   <si>
@@ -208,6 +232,36 @@
     <t>https://taqadistribution.com/addc/ar-ae/business/help-and-support/transfer-and-removal-of-electricity-services</t>
   </si>
   <si>
+    <t>addc/ar-ae/business/locations/branches.report.json</t>
+  </si>
+  <si>
+    <t>["hero-text","cards-support"]</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/locations/branches</t>
+  </si>
+  <si>
+    <t>locations</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:53:02.465Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/locations/branches</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/locations/partners.report.json</t>
+  </si>
+  <si>
+    <t>addc/ar-ae/business/locations/partners</t>
+  </si>
+  <si>
+    <t>2026-09-22T06:53:12.213Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/ar-ae/business/locations/partners</t>
+  </si>
+  <si>
     <t>addc/en-us/business/help-and-support/account-management-and-bills.report.json</t>
   </si>
   <si>
@@ -283,13 +337,7 @@
     <t>addc/en-us/business/locations/branches.report.json</t>
   </si>
   <si>
-    <t>["hero-text","cards-support"]</t>
-  </si>
-  <si>
     <t>addc/en-us/business/locations/branches</t>
-  </si>
-  <si>
-    <t>locations</t>
   </si>
   <si>
     <t>2026-09-22T06:47:20.889Z</t>
@@ -708,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -905,42 +953,42 @@
         <v>43</v>
       </c>
       <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
         <v>44</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
         <v>45</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" t="s">
         <v>46</v>
-      </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" t="s">
-        <v>37</v>
-      </c>
-      <c r="H8" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
         <v>49</v>
       </c>
-      <c r="B9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
         <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>46</v>
       </c>
       <c r="F9" t="s">
         <v>51</v>
@@ -957,7 +1005,7 @@
         <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
         <v>54</v>
@@ -966,7 +1014,7 @@
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F10" t="s">
         <v>55</v>
@@ -983,7 +1031,7 @@
         <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
         <v>58</v>
@@ -992,7 +1040,7 @@
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F11" t="s">
         <v>59</v>
@@ -1009,7 +1057,7 @@
         <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
         <v>62</v>
@@ -1018,7 +1066,7 @@
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F12" t="s">
         <v>63</v>
@@ -1035,7 +1083,7 @@
         <v>65</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
         <v>66</v>
@@ -1044,7 +1092,7 @@
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F13" t="s">
         <v>67</v>
@@ -1061,7 +1109,7 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
         <v>70</v>
@@ -1070,7 +1118,7 @@
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F14" t="s">
         <v>71</v>
@@ -1087,120 +1135,120 @@
         <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G15" t="s">
         <v>37</v>
       </c>
       <c r="H15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
         <v>37</v>
       </c>
       <c r="H16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
         <v>37</v>
       </c>
       <c r="H17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
         <v>37</v>
       </c>
       <c r="H18" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="F19" t="s">
         <v>93</v>
@@ -1217,7 +1265,7 @@
         <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
         <v>96</v>
@@ -1226,7 +1274,7 @@
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="F20" t="s">
         <v>97</v>
@@ -1243,7 +1291,7 @@
         <v>99</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
         <v>100</v>
@@ -1252,7 +1300,7 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F21" t="s">
         <v>101</v>
@@ -1262,6 +1310,110 @@
       </c>
       <c r="H21" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" t="s">
+        <v>105</v>
+      </c>
+      <c r="G22" t="s">
+        <v>37</v>
+      </c>
+      <c r="H22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H23" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" t="s">
+        <v>112</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" t="s">
+        <v>113</v>
+      </c>
+      <c r="G24" t="s">
+        <v>37</v>
+      </c>
+      <c r="H24" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" t="s">
+        <v>116</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" t="s">
+        <v>117</v>
+      </c>
+      <c r="G25" t="s">
+        <v>37</v>
+      </c>
+      <c r="H25" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>